<commit_message>
feat: refresh financial analysis workflow and business data
</commit_message>
<xml_diff>
--- a/docs/data/教育后勤2025经营数据看版_组织标签映射表-勿动.xlsx
+++ b/docs/data/教育后勤2025经营数据看版_组织标签映射表-勿动.xlsx
@@ -10,7 +10,7 @@
     <sheet name="组织标签映射表-勿动" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'组织标签映射表-勿动'!$A$6:$E$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'组织标签映射表-勿动'!$A$1:$D$159</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="186">
   <si>
     <t>level_0</t>
   </si>
@@ -359,7 +359,10 @@
     <t>玉门一中后勤</t>
   </si>
   <si>
-    <t>周口示范区物业</t>
+    <t>周口示范区物业项目</t>
+  </si>
+  <si>
+    <t>修改</t>
   </si>
   <si>
     <t>安全管理平台</t>
@@ -570,6 +573,21 @@
   </si>
   <si>
     <t>后勤数智研发部</t>
+  </si>
+  <si>
+    <t>虎林配送</t>
+  </si>
+  <si>
+    <t>新增</t>
+  </si>
+  <si>
+    <t>亳州地区福利外拓</t>
+  </si>
+  <si>
+    <t>镇沅一中食堂</t>
+  </si>
+  <si>
+    <t>长顺项目本级</t>
   </si>
 </sst>
 </file>
@@ -582,7 +600,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -598,6 +616,24 @@
       <sz val="10"/>
       <name val="Calibri"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="DengXian"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -951,12 +987,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1060,31 +1111,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1093,119 +1132,131 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1213,6 +1264,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1280,6 +1338,11 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="00FF0000"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1546,8 +1609,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D155"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.8" outlineLevelCol="3"/>
+  <dimension ref="A1:F159"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="17.2222222222222" customWidth="1"/>
@@ -2808,7 +2871,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="91" ht="25.5" customHeight="1" spans="1:4">
+    <row r="91" ht="25.5" customHeight="1" spans="1:6">
       <c r="A91" t="s">
         <v>4</v>
       </c>
@@ -2818,8 +2881,14 @@
       <c r="C91" t="s">
         <v>64</v>
       </c>
-      <c r="D91" t="s">
+      <c r="D91" s="5" t="s">
         <v>109</v>
+      </c>
+      <c r="E91" t="s">
+        <v>110</v>
+      </c>
+      <c r="F91">
+        <v>20260407</v>
       </c>
     </row>
     <row r="92" ht="25.5" customHeight="1" spans="1:4">
@@ -2833,7 +2902,7 @@
         <v>48</v>
       </c>
       <c r="D92" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="93" ht="25.5" customHeight="1" spans="1:4">
@@ -2847,7 +2916,7 @@
         <v>30</v>
       </c>
       <c r="D93" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="94" ht="25.5" customHeight="1" spans="1:4">
@@ -2861,7 +2930,7 @@
         <v>30</v>
       </c>
       <c r="D94" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="95" ht="25.5" customHeight="1" spans="1:4">
@@ -2875,7 +2944,7 @@
         <v>30</v>
       </c>
       <c r="D95" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="96" ht="25.5" customHeight="1" spans="1:4">
@@ -2889,7 +2958,7 @@
         <v>30</v>
       </c>
       <c r="D96" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="97" ht="25.5" customHeight="1" spans="1:4">
@@ -2903,7 +2972,7 @@
         <v>30</v>
       </c>
       <c r="D97" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="98" ht="25.5" customHeight="1" spans="1:4">
@@ -2917,7 +2986,7 @@
         <v>30</v>
       </c>
       <c r="D98" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="99" ht="25.5" customHeight="1" spans="1:4">
@@ -2931,7 +3000,7 @@
         <v>36</v>
       </c>
       <c r="D99" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="100" ht="25.5" customHeight="1" spans="1:4">
@@ -2945,7 +3014,7 @@
         <v>36</v>
       </c>
       <c r="D100" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="101" ht="25.5" customHeight="1" spans="1:4">
@@ -2959,7 +3028,7 @@
         <v>36</v>
       </c>
       <c r="D101" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="102" ht="25.5" customHeight="1" spans="1:4">
@@ -2973,7 +3042,7 @@
         <v>36</v>
       </c>
       <c r="D102" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="103" ht="25.5" customHeight="1" spans="1:4">
@@ -2987,7 +3056,7 @@
         <v>36</v>
       </c>
       <c r="D103" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="104" ht="25.5" customHeight="1" spans="1:4">
@@ -3001,7 +3070,7 @@
         <v>36</v>
       </c>
       <c r="D104" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="105" ht="25.5" customHeight="1" spans="1:4">
@@ -3015,7 +3084,7 @@
         <v>36</v>
       </c>
       <c r="D105" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="106" ht="25.5" customHeight="1" spans="1:4">
@@ -3029,7 +3098,7 @@
         <v>36</v>
       </c>
       <c r="D106" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="107" ht="25.5" customHeight="1" spans="1:4">
@@ -3043,7 +3112,7 @@
         <v>36</v>
       </c>
       <c r="D107" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="108" ht="25.5" customHeight="1" spans="1:4">
@@ -3057,7 +3126,7 @@
         <v>43</v>
       </c>
       <c r="D108" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="109" ht="25.5" customHeight="1" spans="1:4">
@@ -3071,7 +3140,7 @@
         <v>43</v>
       </c>
       <c r="D109" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="110" ht="25.5" customHeight="1" spans="1:4">
@@ -3085,7 +3154,7 @@
         <v>43</v>
       </c>
       <c r="D110" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="111" ht="25.5" customHeight="1" spans="1:4">
@@ -3099,7 +3168,7 @@
         <v>43</v>
       </c>
       <c r="D111" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="112" ht="25.5" customHeight="1" spans="1:4">
@@ -3113,7 +3182,7 @@
         <v>43</v>
       </c>
       <c r="D112" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="113" ht="25.5" customHeight="1" spans="1:4">
@@ -3127,7 +3196,7 @@
         <v>64</v>
       </c>
       <c r="D113" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="114" ht="25.5" customHeight="1" spans="1:4">
@@ -3141,7 +3210,7 @@
         <v>64</v>
       </c>
       <c r="D114" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="115" ht="25.5" customHeight="1" spans="1:4">
@@ -3155,7 +3224,7 @@
         <v>64</v>
       </c>
       <c r="D115" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="116" ht="25.5" customHeight="1" spans="1:4">
@@ -3169,7 +3238,7 @@
         <v>48</v>
       </c>
       <c r="D116" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="117" ht="25.5" customHeight="1" spans="1:4">
@@ -3183,7 +3252,7 @@
         <v>48</v>
       </c>
       <c r="D117" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="118" ht="25.5" customHeight="1" spans="1:4">
@@ -3197,7 +3266,7 @@
         <v>48</v>
       </c>
       <c r="D118" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="119" ht="25.5" customHeight="1" spans="1:4">
@@ -3211,7 +3280,7 @@
         <v>48</v>
       </c>
       <c r="D119" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="120" ht="25.5" customHeight="1" spans="1:4">
@@ -3225,7 +3294,7 @@
         <v>75</v>
       </c>
       <c r="D120" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="121" s="2" customFormat="1" ht="25.5" customHeight="1" spans="1:4">
@@ -3233,13 +3302,13 @@
         <v>4</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="122" ht="25.5" customHeight="1" spans="1:4">
@@ -3247,13 +3316,13 @@
         <v>4</v>
       </c>
       <c r="B122" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C122" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D122" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="123" ht="25.5" customHeight="1" spans="1:4">
@@ -3261,13 +3330,13 @@
         <v>4</v>
       </c>
       <c r="B123" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C123" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D123" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="124" ht="25.5" customHeight="1" spans="1:4">
@@ -3275,13 +3344,13 @@
         <v>4</v>
       </c>
       <c r="B124" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C124" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D124" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="125" ht="25.5" customHeight="1" spans="1:4">
@@ -3289,13 +3358,13 @@
         <v>4</v>
       </c>
       <c r="B125" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C125" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D125" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="126" ht="25.5" customHeight="1" spans="1:4">
@@ -3303,13 +3372,13 @@
         <v>4</v>
       </c>
       <c r="B126" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C126" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D126" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="127" ht="25.5" customHeight="1" spans="1:4">
@@ -3317,13 +3386,13 @@
         <v>4</v>
       </c>
       <c r="B127" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C127" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D127" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="128" ht="25.5" customHeight="1" spans="1:4">
@@ -3331,13 +3400,13 @@
         <v>4</v>
       </c>
       <c r="B128" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C128" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D128" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="129" ht="25.5" customHeight="1" spans="1:4">
@@ -3345,13 +3414,13 @@
         <v>4</v>
       </c>
       <c r="B129" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C129" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D129" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="130" ht="25.5" customHeight="1" spans="1:4">
@@ -3359,13 +3428,13 @@
         <v>4</v>
       </c>
       <c r="B130" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C130" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D130" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="131" ht="25.5" customHeight="1" spans="1:4">
@@ -3373,13 +3442,13 @@
         <v>4</v>
       </c>
       <c r="B131" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C131" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D131" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="132" ht="25.5" customHeight="1" spans="1:4">
@@ -3387,13 +3456,13 @@
         <v>4</v>
       </c>
       <c r="B132" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C132" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D132" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="133" ht="25.5" customHeight="1" spans="1:4">
@@ -3401,13 +3470,13 @@
         <v>4</v>
       </c>
       <c r="B133" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C133" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D133" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="134" ht="25.5" customHeight="1" spans="1:4">
@@ -3415,13 +3484,13 @@
         <v>4</v>
       </c>
       <c r="B134" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C134" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D134" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="135" ht="25.5" customHeight="1" spans="1:4">
@@ -3429,13 +3498,13 @@
         <v>4</v>
       </c>
       <c r="B135" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C135" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D135" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="136" ht="25.5" customHeight="1" spans="1:4">
@@ -3443,13 +3512,13 @@
         <v>4</v>
       </c>
       <c r="B136" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C136" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D136" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="137" ht="25.5" customHeight="1" spans="1:4">
@@ -3457,13 +3526,13 @@
         <v>4</v>
       </c>
       <c r="B137" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C137" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D137" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="138" ht="25.5" customHeight="1" spans="1:4">
@@ -3471,13 +3540,13 @@
         <v>4</v>
       </c>
       <c r="B138" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C138" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D138" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="139" ht="25.5" customHeight="1" spans="1:4">
@@ -3485,13 +3554,13 @@
         <v>4</v>
       </c>
       <c r="B139" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C139" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D139" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="140" ht="25.5" customHeight="1" spans="1:4">
@@ -3499,13 +3568,13 @@
         <v>4</v>
       </c>
       <c r="B140" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C140" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D140" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="141" ht="25.5" customHeight="1" spans="1:4">
@@ -3513,13 +3582,13 @@
         <v>4</v>
       </c>
       <c r="B141" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C141" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D141" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="142" ht="25.5" customHeight="1" spans="1:4">
@@ -3527,13 +3596,13 @@
         <v>4</v>
       </c>
       <c r="B142" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C142" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D142" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="143" ht="25.5" customHeight="1" spans="1:4">
@@ -3541,13 +3610,13 @@
         <v>4</v>
       </c>
       <c r="B143" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C143" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D143" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="144" ht="25.5" customHeight="1" spans="1:4">
@@ -3555,13 +3624,13 @@
         <v>4</v>
       </c>
       <c r="B144" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C144" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D144" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="145" ht="25.5" customHeight="1" spans="1:4">
@@ -3569,13 +3638,13 @@
         <v>4</v>
       </c>
       <c r="B145" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C145" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D145" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="146" ht="25.5" customHeight="1" spans="1:4">
@@ -3583,10 +3652,10 @@
         <v>4</v>
       </c>
       <c r="B146" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D146" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="147" ht="25.5" customHeight="1" spans="1:4">
@@ -3594,10 +3663,10 @@
         <v>4</v>
       </c>
       <c r="B147" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D147" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="148" ht="25.5" customHeight="1" spans="1:4">
@@ -3605,10 +3674,10 @@
         <v>4</v>
       </c>
       <c r="B148" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D148" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="149" ht="25.5" customHeight="1" spans="1:4">
@@ -3616,10 +3685,10 @@
         <v>4</v>
       </c>
       <c r="B149" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D149" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="150" ht="25.5" customHeight="1" spans="1:4">
@@ -3627,10 +3696,10 @@
         <v>4</v>
       </c>
       <c r="B150" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D150" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="151" ht="25.5" customHeight="1" spans="1:4">
@@ -3638,10 +3707,10 @@
         <v>4</v>
       </c>
       <c r="B151" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D151" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="152" ht="25.5" customHeight="1" spans="1:4">
@@ -3649,10 +3718,10 @@
         <v>4</v>
       </c>
       <c r="B152" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D152" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="153" ht="25.5" customHeight="1" spans="1:4">
@@ -3660,10 +3729,10 @@
         <v>4</v>
       </c>
       <c r="B153" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D153" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="154" ht="25.5" customHeight="1" spans="1:4">
@@ -3671,10 +3740,10 @@
         <v>4</v>
       </c>
       <c r="B154" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D154" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="155" ht="25.5" customHeight="1" spans="1:4">
@@ -3682,27 +3751,107 @@
         <v>4</v>
       </c>
       <c r="B155" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D155" t="s">
-        <v>179</v>
+        <v>180</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6">
+      <c r="A156" t="s">
+        <v>4</v>
+      </c>
+      <c r="B156" t="s">
+        <v>99</v>
+      </c>
+      <c r="C156" t="s">
+        <v>30</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E156" t="s">
+        <v>182</v>
+      </c>
+      <c r="F156">
+        <v>20260407</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6">
+      <c r="A157" t="s">
+        <v>4</v>
+      </c>
+      <c r="B157" t="s">
+        <v>77</v>
+      </c>
+      <c r="C157" t="s">
+        <v>43</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E157" t="s">
+        <v>182</v>
+      </c>
+      <c r="F157">
+        <v>20260407</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6">
+      <c r="A158" t="s">
+        <v>4</v>
+      </c>
+      <c r="B158" t="s">
+        <v>29</v>
+      </c>
+      <c r="C158" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D158" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="E158" t="s">
+        <v>182</v>
+      </c>
+      <c r="F158">
+        <v>20260407</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6">
+      <c r="A159" t="s">
+        <v>4</v>
+      </c>
+      <c r="B159" t="s">
+        <v>29</v>
+      </c>
+      <c r="C159" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D159" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="E159" t="s">
+        <v>182</v>
+      </c>
+      <c r="F159">
+        <v>20260407</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D159" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
+  <conditionalFormatting sqref="D$1:D$1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" sqref="B2:B19 B121:B154">
       <formula1>"后勤管理中心,三大区域,商业业务,科创发展中心,战略支持中心,后勤集团总裁室"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="B20:B120 C2:C19 C121:C154">
+    <dataValidation type="list" sqref="B20:B120 B156:B157 C2:C19 C121:C154">
       <formula1>"教育园特色餐饮,念心湖酒店,海亮后勤车队,海亮医院,中心其余业务部门,中心管理部门,西南区域,东部区域,北部区域,战略支持中心,商超业务-便利店,商超业务-商业街,科创发展中心,线下商超-便利店,线上商城业务,后勤集团总裁室,线下商超-商业街,融爱星餐饮"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C20:C120">
+    <dataValidation type="list" sqref="C20:C120 C156:C157">
       <formula1>"区域配送业务,区域餐饮业务,区域商超业务,区域物业业务,区域科技业务,区域总经理室,线下便利店,线上商城,中心餐饮业务,中心物业业务,其他,管理部门,线下商业街"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update opportunity snapshot UI and data workflows
</commit_message>
<xml_diff>
--- a/docs/data/教育后勤2025经营数据看版_组织标签映射表-勿动.xlsx
+++ b/docs/data/教育后勤2025经营数据看版_组织标签映射表-勿动.xlsx
@@ -10,7 +10,7 @@
     <sheet name="组织标签映射表-勿动" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'组织标签映射表-勿动'!$A$1:$D$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'组织标签映射表-勿动'!$A$1:$F$159</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="184">
   <si>
     <t>level_0</t>
   </si>
@@ -452,16 +452,16 @@
     <t>北部区域总经理室</t>
   </si>
   <si>
+    <t>科创发展中心</t>
+  </si>
+  <si>
     <t>商业业务</t>
   </si>
   <si>
-    <t>管理部门</t>
-  </si>
-  <si>
     <t>后勤数智零售部</t>
   </si>
   <si>
-    <t>线下商超-便利店</t>
+    <t>0421修改映射</t>
   </si>
   <si>
     <t>皓峰初中店</t>
@@ -515,9 +515,6 @@
     <t>宁海公学文创店</t>
   </si>
   <si>
-    <t>线下商超-商业街</t>
-  </si>
-  <si>
     <t>海实文创店</t>
   </si>
   <si>
@@ -558,9 +555,6 @@
   </si>
   <si>
     <t>后勤集团总裁室</t>
-  </si>
-  <si>
-    <t>科创发展中心</t>
   </si>
   <si>
     <t>托管学校入模产品服务</t>
@@ -787,7 +781,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -797,6 +791,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1132,7 +1132,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1156,16 +1156,16 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1174,89 +1174,89 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1267,6 +1267,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -3297,354 +3298,429 @@
         <v>139</v>
       </c>
     </row>
-    <row r="121" s="2" customFormat="1" ht="25.5" customHeight="1" spans="1:4">
+    <row r="121" s="2" customFormat="1" ht="25.5" customHeight="1" spans="1:5">
       <c r="A121" t="s">
         <v>4</v>
       </c>
-      <c r="B121" s="2" t="s">
+      <c r="B121" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C121" s="2" t="s">
+      <c r="C121" s="6" t="s">
         <v>141</v>
       </c>
       <c r="D121" s="2" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="122" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E121" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="122" ht="25.5" customHeight="1" spans="1:5">
       <c r="A122" t="s">
         <v>4</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C122" t="s">
-        <v>143</v>
+      <c r="C122" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D122" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="123" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E122" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="123" ht="25.5" customHeight="1" spans="1:5">
       <c r="A123" t="s">
         <v>4</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C123" t="s">
-        <v>143</v>
+      <c r="C123" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D123" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="124" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E123" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="124" ht="25.5" customHeight="1" spans="1:5">
       <c r="A124" t="s">
         <v>4</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C124" t="s">
-        <v>143</v>
+      <c r="C124" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D124" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="125" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E124" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="125" ht="25.5" customHeight="1" spans="1:5">
       <c r="A125" t="s">
         <v>4</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C125" t="s">
-        <v>143</v>
+      <c r="C125" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D125" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="126" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E125" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="126" ht="25.5" customHeight="1" spans="1:5">
       <c r="A126" t="s">
         <v>4</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C126" t="s">
-        <v>143</v>
+      <c r="C126" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D126" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="127" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E126" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="127" ht="25.5" customHeight="1" spans="1:5">
       <c r="A127" t="s">
         <v>4</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C127" t="s">
-        <v>143</v>
+      <c r="C127" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D127" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="128" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E127" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="128" ht="25.5" customHeight="1" spans="1:5">
       <c r="A128" t="s">
         <v>4</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C128" t="s">
-        <v>143</v>
+      <c r="C128" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D128" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="129" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E128" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="129" ht="25.5" customHeight="1" spans="1:5">
       <c r="A129" t="s">
         <v>4</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C129" t="s">
-        <v>143</v>
+      <c r="C129" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D129" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="130" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E129" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="130" ht="25.5" customHeight="1" spans="1:5">
       <c r="A130" t="s">
         <v>4</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C130" t="s">
-        <v>143</v>
+      <c r="C130" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D130" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="131" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E130" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="131" ht="25.5" customHeight="1" spans="1:5">
       <c r="A131" t="s">
         <v>4</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C131" t="s">
-        <v>143</v>
+      <c r="C131" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D131" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="132" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E131" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="132" ht="25.5" customHeight="1" spans="1:5">
       <c r="A132" t="s">
         <v>4</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C132" t="s">
-        <v>143</v>
+      <c r="C132" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D132" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="133" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E132" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="133" ht="25.5" customHeight="1" spans="1:5">
       <c r="A133" t="s">
         <v>4</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C133" t="s">
-        <v>143</v>
+      <c r="C133" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D133" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="134" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E133" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="134" ht="25.5" customHeight="1" spans="1:5">
       <c r="A134" t="s">
         <v>4</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C134" t="s">
-        <v>143</v>
+      <c r="C134" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D134" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="135" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E134" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="135" ht="25.5" customHeight="1" spans="1:5">
       <c r="A135" t="s">
         <v>4</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C135" t="s">
-        <v>143</v>
+      <c r="C135" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D135" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="136" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E135" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="136" ht="25.5" customHeight="1" spans="1:5">
       <c r="A136" t="s">
         <v>4</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B136" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C136" t="s">
-        <v>143</v>
+      <c r="C136" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D136" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="137" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E136" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="137" ht="25.5" customHeight="1" spans="1:5">
       <c r="A137" t="s">
         <v>4</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B137" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C137" t="s">
-        <v>143</v>
+      <c r="C137" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D137" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="138" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E137" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="138" ht="25.5" customHeight="1" spans="1:5">
       <c r="A138" t="s">
         <v>4</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B138" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C138" t="s">
-        <v>143</v>
+      <c r="C138" s="6" t="s">
+        <v>141</v>
       </c>
       <c r="D138" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="139" ht="25.5" customHeight="1" spans="1:4">
+      <c r="E138" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="139" ht="25.5" customHeight="1" spans="1:5">
       <c r="A139" t="s">
         <v>4</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B139" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C139" t="s">
+      <c r="C139" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D139" t="s">
         <v>161</v>
       </c>
-      <c r="D139" t="s">
+      <c r="E139" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="140" ht="25.5" customHeight="1" spans="1:5">
+      <c r="A140" t="s">
+        <v>4</v>
+      </c>
+      <c r="B140" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C140" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D140" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="140" ht="25.5" customHeight="1" spans="1:4">
-      <c r="A140" t="s">
-        <v>4</v>
-      </c>
-      <c r="B140" t="s">
+      <c r="E140" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="141" ht="25.5" customHeight="1" spans="1:5">
+      <c r="A141" t="s">
+        <v>4</v>
+      </c>
+      <c r="B141" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C140" t="s">
-        <v>161</v>
-      </c>
-      <c r="D140" t="s">
+      <c r="C141" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D141" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="141" ht="25.5" customHeight="1" spans="1:4">
-      <c r="A141" t="s">
-        <v>4</v>
-      </c>
-      <c r="B141" t="s">
+      <c r="E141" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="142" ht="25.5" customHeight="1" spans="1:5">
+      <c r="A142" t="s">
+        <v>4</v>
+      </c>
+      <c r="B142" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C141" t="s">
-        <v>161</v>
-      </c>
-      <c r="D141" t="s">
+      <c r="C142" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D142" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="142" ht="25.5" customHeight="1" spans="1:4">
-      <c r="A142" t="s">
-        <v>4</v>
-      </c>
-      <c r="B142" t="s">
+      <c r="E142" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="143" ht="25.5" customHeight="1" spans="1:5">
+      <c r="A143" t="s">
+        <v>4</v>
+      </c>
+      <c r="B143" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C142" t="s">
-        <v>161</v>
-      </c>
-      <c r="D142" t="s">
+      <c r="C143" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D143" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="143" ht="25.5" customHeight="1" spans="1:4">
-      <c r="A143" t="s">
-        <v>4</v>
-      </c>
-      <c r="B143" t="s">
+      <c r="E143" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="144" ht="25.5" customHeight="1" spans="1:5">
+      <c r="A144" t="s">
+        <v>4</v>
+      </c>
+      <c r="B144" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C143" t="s">
-        <v>161</v>
-      </c>
-      <c r="D143" t="s">
+      <c r="C144" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D144" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="144" ht="25.5" customHeight="1" spans="1:4">
-      <c r="A144" t="s">
-        <v>4</v>
-      </c>
-      <c r="B144" t="s">
+      <c r="E144" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="145" ht="25.5" customHeight="1" spans="1:5">
+      <c r="A145" t="s">
+        <v>4</v>
+      </c>
+      <c r="B145" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C144" t="s">
-        <v>161</v>
-      </c>
-      <c r="D144" t="s">
+      <c r="C145" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D145" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="145" ht="25.5" customHeight="1" spans="1:4">
-      <c r="A145" t="s">
-        <v>4</v>
-      </c>
-      <c r="B145" t="s">
-        <v>140</v>
-      </c>
-      <c r="C145" t="s">
-        <v>168</v>
-      </c>
-      <c r="D145" t="s">
-        <v>168</v>
+      <c r="E145" s="6" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="146" ht="25.5" customHeight="1" spans="1:4">
@@ -3652,10 +3728,10 @@
         <v>4</v>
       </c>
       <c r="B146" t="s">
+        <v>168</v>
+      </c>
+      <c r="D146" t="s">
         <v>169</v>
-      </c>
-      <c r="D146" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="147" ht="25.5" customHeight="1" spans="1:4">
@@ -3663,10 +3739,10 @@
         <v>4</v>
       </c>
       <c r="B147" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D147" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="148" ht="25.5" customHeight="1" spans="1:4">
@@ -3674,10 +3750,10 @@
         <v>4</v>
       </c>
       <c r="B148" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D148" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="149" ht="25.5" customHeight="1" spans="1:4">
@@ -3685,10 +3761,10 @@
         <v>4</v>
       </c>
       <c r="B149" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D149" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="150" ht="25.5" customHeight="1" spans="1:4">
@@ -3696,10 +3772,10 @@
         <v>4</v>
       </c>
       <c r="B150" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D150" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="151" ht="25.5" customHeight="1" spans="1:4">
@@ -3707,10 +3783,10 @@
         <v>4</v>
       </c>
       <c r="B151" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D151" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="152" ht="25.5" customHeight="1" spans="1:4">
@@ -3718,10 +3794,10 @@
         <v>4</v>
       </c>
       <c r="B152" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="D152" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="153" ht="25.5" customHeight="1" spans="1:4">
@@ -3729,10 +3805,10 @@
         <v>4</v>
       </c>
       <c r="B153" t="s">
+        <v>140</v>
+      </c>
+      <c r="D153" t="s">
         <v>176</v>
-      </c>
-      <c r="D153" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="154" ht="25.5" customHeight="1" spans="1:4">
@@ -3740,10 +3816,10 @@
         <v>4</v>
       </c>
       <c r="B154" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="D154" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="155" ht="25.5" customHeight="1" spans="1:4">
@@ -3751,10 +3827,10 @@
         <v>4</v>
       </c>
       <c r="B155" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="D155" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -3768,10 +3844,10 @@
         <v>30</v>
       </c>
       <c r="D156" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E156" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F156">
         <v>20260407</v>
@@ -3788,10 +3864,10 @@
         <v>43</v>
       </c>
       <c r="D157" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E157" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F157">
         <v>20260407</v>
@@ -3804,14 +3880,14 @@
       <c r="B158" t="s">
         <v>29</v>
       </c>
-      <c r="C158" s="6" t="s">
+      <c r="C158" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D158" s="7" t="s">
-        <v>184</v>
+      <c r="D158" s="8" t="s">
+        <v>182</v>
       </c>
       <c r="E158" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F158">
         <v>20260407</v>
@@ -3824,31 +3900,31 @@
       <c r="B159" t="s">
         <v>29</v>
       </c>
-      <c r="C159" s="6" t="s">
+      <c r="C159" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D159" s="7" t="s">
-        <v>185</v>
+      <c r="D159" s="8" t="s">
+        <v>183</v>
       </c>
       <c r="E159" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F159">
         <v>20260407</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D159" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:F159" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="D$1:D$1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" sqref="B2:B19 B121:B154">
+    <dataValidation type="list" sqref="B2:B19 B121:B154 C121:C145">
       <formula1>"后勤管理中心,三大区域,商业业务,科创发展中心,战略支持中心,后勤集团总裁室"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="B20:B120 B156:B157 C2:C19 C121:C154">
+    <dataValidation type="list" sqref="B20:B120 B156:B157 C2:C19 C146:C154">
       <formula1>"教育园特色餐饮,念心湖酒店,海亮后勤车队,海亮医院,中心其余业务部门,中心管理部门,西南区域,东部区域,北部区域,战略支持中心,商超业务-便利店,商超业务-商业街,科创发展中心,线下商超-便利店,线上商城业务,后勤集团总裁室,线下商超-商业街,融爱星餐饮"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="C20:C120 C156:C157">

</xml_diff>